<commit_message>
Finished unit test cases for the dunder init for ChequingAccount subclass.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rrcca-my.sharepoint.com/personal/emaglaque2_rrc_ca/Documents/Documents/rrc-polytech/term-2/intermediate-software-comp-2327/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D81FC1E-46C7-4B56-A4CB-D6B041271170}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BF4ED52-CFC1-4468-BD4B-1C87A549B762}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
@@ -269,12 +269,6 @@
     <t xml:space="preserve">date_created = today's date </t>
   </si>
   <si>
-    <t>service_charge = 0.50</t>
-  </si>
-  <si>
-    <t>service_charge = 25.50</t>
-  </si>
-  <si>
     <t>444, 200304, 0,
 "invalid", -100, 0.05</t>
   </si>
@@ -286,29 +280,35 @@
 Overdraft limit: $-100 Overdraft Rate: 5.00% Account Type: Chequing"</t>
   </si>
   <si>
+    <t>service_charge = $0.50</t>
+  </si>
+  <si>
+    <t>service_charge = $25.50</t>
+  </si>
+  <si>
     <t>444, 200304, 0,
-date(2020, 12, 4), -100, 0.05</t>
+date.today(), -100, 0.05</t>
   </si>
   <si>
     <t>444, 200304, 0,
-date(2020, 12, 4), "invalid", 0.05</t>
+date.today(), "invalid", 0.05</t>
   </si>
   <si>
     <t>444, 200304, 0,
-date(2020, 12, 4), -100, "invalid"</t>
+date.today(), -100, "invalid"</t>
   </si>
   <si>
     <t>ChequingAccount(444, 200304, 0,
-date(2020, 12, 4), -100, 0.05)</t>
+date.today(), -100, 0.05)</t>
   </si>
   <si>
     <t>ChequingAccount(444, 200304, 0,
-date(2020, 12, 4), -100, 0.05)
+date.today(), -100, 0.05)
 self.__balance = -600</t>
   </si>
   <si>
     <t>ChequingAccount(444, 200304, 0,
-date(2020, 12, 4), -100, 0.05)
+date.today(), -100, 0.05)
 self.__balance = -100</t>
   </si>
 </sst>
@@ -1278,7 +1278,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>22</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G10" s="13" t="s">
         <v>27</v>
@@ -1372,13 +1372,13 @@
         <v>36</v>
       </c>
       <c r="F11" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="2:7" ht="43.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1392,10 +1392,10 @@
         <v>37</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1412,10 +1412,10 @@
         <v>38</v>
       </c>
       <c r="F13" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="13" t="s">
         <v>31</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1435,7 +1435,7 @@
         <v>22</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Finished all of the unit tests for ChequingAccount subclass.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rrcca-my.sharepoint.com/personal/emaglaque2_rrc_ca/Documents/Documents/rrc-polytech/term-2/intermediate-software-comp-2327/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BF4ED52-CFC1-4468-BD4B-1C87A549B762}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B81E03C-FC83-4C47-AC35-E48DB4E2BD53}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
@@ -276,16 +276,6 @@
     <t>ChequingAccount object from preconditions</t>
   </si>
   <si>
-    <t>"Account Number: 444 Balance: $0\n 
-Overdraft limit: $-100 Overdraft Rate: 5.00% Account Type: Chequing"</t>
-  </si>
-  <si>
-    <t>service_charge = $0.50</t>
-  </si>
-  <si>
-    <t>service_charge = $25.50</t>
-  </si>
-  <si>
     <t>444, 200304, 0,
 date.today(), -100, 0.05</t>
   </si>
@@ -310,6 +300,16 @@
     <t>ChequingAccount(444, 200304, 0,
 date.today(), -100, 0.05)
 self.__balance = -100</t>
+  </si>
+  <si>
+    <t>service_charge = 0.50</t>
+  </si>
+  <si>
+    <t>service_charge = 25.50</t>
+  </si>
+  <si>
+    <t>"Account Number: 444 Balance: $0.00\n 
+Overdraft Limit: $-100.00 Overdraft Rate: 5.00% Account Type: Chequing"</t>
   </si>
 </sst>
 </file>
@@ -1292,7 +1292,7 @@
         <v>22</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>24</v>
@@ -1312,7 +1312,7 @@
         <v>22</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>25</v>
@@ -1332,7 +1332,7 @@
         <v>22</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>26</v>
@@ -1369,13 +1369,13 @@
         <v>14</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="43.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1389,13 +1389,13 @@
         <v>18</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1409,13 +1409,13 @@
         <v>19</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1429,13 +1429,13 @@
         <v>20</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>22</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Made InvestmentAccount subclass and finished __init__ implementation.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rrcca-my.sharepoint.com/personal/emaglaque2_rrc_ca/Documents/Documents/rrc-polytech/term-2/intermediate-software-comp-2327/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B81E03C-FC83-4C47-AC35-E48DB4E2BD53}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A3F22B4-998C-438E-82C6-E129A605EE5C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
@@ -1378,7 +1378,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="43.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>6</v>
       </c>

</xml_diff>